<commit_message>
Restore BMP and CMU access list
</commit_message>
<xml_diff>
--- a/Daftar_Akses_Portal.xlsx
+++ b/Daftar_Akses_Portal.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,814 +441,2002 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>80002118.0</t>
+          <t>1611241</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>JOHANSYAH</t>
+          <t>AHMAD FADHOLI</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3314VX</t>
+          <t>1K9BNO</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>80001861.0</t>
+          <t>1508261</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AL FAIZAL WIJAYA</t>
+          <t>AHMAD FIRDAUS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>L0O0RT</t>
+          <t>YGZXHU</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>80002120.0</t>
+          <t>2006251</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MUHAMMAD SAID</t>
+          <t>AHMAD JURDI</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PKXJQA</t>
+          <t>0HP357</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>80002253.0</t>
+          <t>1102261</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SUPRIADI</t>
+          <t>AHMAD KURNIAWAN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7J6J78</t>
+          <t>BR1Z1V</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>80003010.0</t>
+          <t>2804232</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TAUFIK HIDAYAT</t>
+          <t>AHMAD NOR</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>9VGCO8</t>
+          <t>J3R7FW</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>80003132.0</t>
+          <t>2802253</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BALINTON SITEPU</t>
+          <t>AHMAD YUNUS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1P3YT3</t>
+          <t>51TXBL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>80004079.0</t>
+          <t>207251</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RUSLI</t>
+          <t>AHMAT SUGIANOR</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>WTANQT</t>
+          <t>7BUQ6H</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>80004296.0</t>
+          <t>2910241</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>HERI PORWANTO</t>
+          <t>ALDO WARTA SAPUTRA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CZEXPS</t>
+          <t>WB5J2Q</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>80005321.0</t>
+          <t>206231</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>HENDRA GUNAWAN</t>
+          <t>AMANDA MARINDO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>M91234</t>
+          <t>1RQMEM</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>80007180.0</t>
+          <t>201261</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>EKO NURYONO</t>
+          <t>AMINAL HUSNADI</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2T8QZD</t>
+          <t>UF2UCN</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>80007834.0</t>
+          <t>200509251</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ABDUL  SALAM</t>
+          <t>ANDRE JEVISCA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>U9KSS4</t>
+          <t>8L0DSD</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>80008812.0</t>
+          <t>2405261</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PENGKY ANGGARY</t>
+          <t>BUDIMAN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>A0ZKHB</t>
+          <t>7E4M6A</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>80009577.0</t>
+          <t>2405262</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MARDI ARYANTO</t>
+          <t>DAFRIT TIERO BERNANDO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>D5IRWX</t>
+          <t>E40PMD</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>80009581.0</t>
+          <t>202809251</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PARDIANSAH</t>
+          <t>DENIS DAMARA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CLOMD8</t>
+          <t>678Q9B</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>80009701.0</t>
+          <t>1706261</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>IRMAYADI</t>
+          <t>DWIKY RYAMIZARDIN</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6JIT3C</t>
+          <t>FZMSCA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>80013827.0</t>
+          <t>207231</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KORINTUS DEPIN</t>
+          <t>FAJAR PILIPUS SIHOMBING</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>G0SJGC</t>
+          <t>FQQQLB</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>80014093.0</t>
+          <t>1402231</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DANI DWI ADI RAHMADANA</t>
+          <t>HANSO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>XXZYFR</t>
+          <t>HAKR86</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>80014094.0</t>
+          <t>603222</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GATOT PRINGGO SUKOCO</t>
+          <t>IRFAN NURHADI</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>JLXDOH</t>
+          <t>Y4SQ2F</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>80014095.0</t>
+          <t>2802252</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>HERMAWAN DWI SUPRIYADI</t>
+          <t>JIMI ARNOLDY</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ZXRPUE</t>
+          <t>4FYGP2</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>80014153.0</t>
+          <t>1004253</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>FERY GUNAWAN</t>
+          <t>JUMILIN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0EEVMC</t>
+          <t>W3URY8</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>80014154.0</t>
+          <t>200811251</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GIGIH SUTANTO</t>
+          <t>KOMOK</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>YDPLY8</t>
+          <t>P8MYMB</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>80014155.0</t>
+          <t>1508264</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>HERI PRASETYO</t>
+          <t>LEWIS PRISTIANDI</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GY1R12</t>
+          <t>Z70QTI</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>80017427.0</t>
+          <t>1004254</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>RESAL</t>
+          <t>LUTFY YAZID</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NZ844Q</t>
+          <t>S4N7XE</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>80017430.0</t>
+          <t>201409251</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>KORINTUS DEPIN</t>
+          <t>MILKANSYAH</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>LCVLS4</t>
+          <t>8CNH9L</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>80002654.0</t>
+          <t>1906253</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>YONATAN</t>
+          <t>MUHAMMAD AKHSANUL HUDA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NES171</t>
+          <t>BFWR4X</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>80003140.0</t>
+          <t>1510243</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>WANDRA PRIMA PERA</t>
+          <t>MUHAMMAD HUSNI THAMRIN</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>A0CAWT</t>
+          <t>ILHHJQ</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>80004479.0</t>
+          <t>1912241</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GARANTO GURITNO</t>
+          <t>MUHAMMAD ISNUHONI</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NCWWZI</t>
+          <t>XDVMX7</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>80004593.0</t>
+          <t>1508262</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>M ARJUNI</t>
+          <t>MUHAMMAD REFFY FAHREZA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>US26BM</t>
+          <t>KGWMIV</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>80006801.0</t>
+          <t>1508263</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AHMAD ANUGRAH MUFTI ALAM</t>
+          <t>MUHAMMAD RIDWAN</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Y1SS7T</t>
+          <t>U4FN6X</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>80008416.0</t>
+          <t>202809252</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AGUS</t>
+          <t>MUHAMMAD RIZKI FIRDAUS</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>107G0E</t>
+          <t>7LN4FQ</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>80008803.0</t>
+          <t>2604251</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>RINTO PARULIAN SITANGGANG</t>
+          <t>MUHAMMAD ZAINI</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>BG0KFF</t>
+          <t>4AP7EV</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>80009720.0</t>
+          <t>1510241</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>YASER ARAFAT</t>
+          <t>NANDA RIZKY BUDIANTO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>VU7UKL</t>
+          <t>I6BLSG</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>80011723.0</t>
+          <t>2307261</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MUHAMMAD MAHYUDDIN</t>
+          <t>NOVARI FADLI</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0K3I52</t>
+          <t>KT99D2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>80013760.0</t>
+          <t>110241</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>RESAL</t>
+          <t>NOVITA FITRI</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>J87H3C</t>
+          <t>R2Q617</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>80016561.0</t>
+          <t>2703251</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>WAHYU</t>
+          <t>PIGAR</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>SI4FA5</t>
+          <t>L7YPJZ</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>80016612.0</t>
+          <t>108235</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LIANSYAH</t>
+          <t>RANDI</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>9U9TLO</t>
+          <t>DJA5LQ</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>80017177.0</t>
+          <t>1705261</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
+          <t>RESKI</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>MAT0H2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1906252</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>REVALDHY NARADA PUTRA</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>1Z26XJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>108238</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>RIFKY JANUARTA</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>B2DL5W</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>201409252</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ROSID WASKITO</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>DRRBLH</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1507261</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>SERBIANTO</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>W923CF</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1303221</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SUGIANOR</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>QEB2WZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2107261</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SYARIFUDIN</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>I251M4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1004255</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>TEDY SAPUTRA</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>P6KJ80</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2103223</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>THANTAWI FADILAH</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>9K39E9</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>200509255</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>UKANDRI</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>MWK2WV</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>207253</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>VRIO AGUSTINUS</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>S80MHI</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2106234</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>WILDAN IRGIE FAZIRA</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>3R8RZT</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1906254</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ZAINAL HAKIM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>HM3CQA</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>102111001</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>IZAH</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>4W2UHC</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>202311002</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MADRI YANI</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>WUZDRH</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>102311001</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>RISWANDI</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>3X4277</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>102401001</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>TAUFIK KURAHMAN</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>S5EW86</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>10151021</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>YOKO</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>NLMJ9I</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>80007834</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ABDUL  SALAM</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>U9KSS4</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>80008416</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>AGUS</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>107G0E</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>80006801</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>AHMAD ANUGRAH MUFTI ALAM</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Y1SS7T</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>80001861</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>AL FAIZAL WIJAYA</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>L0O0RT</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>80003132</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>BALINTON SITEPU</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1P3YT3</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>80014093</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>DANI DWI ADI RAHMADANA</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>XXZYFR</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>80007180</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>EKO NURYONO</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>2T8QZD</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>80014153</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>FERY GUNAWAN</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>0EEVMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>80004479</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>GARANTO GURITNO</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>NCWWZI</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>80014094</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>GATOT PRINGGO SUKOCO</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>JLXDOH</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>80014154</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>GIGIH SUTANTO</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>YDPLY8</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>80005321</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>HENDRA GUNAWAN</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>M91234</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>80004296</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>HERI PORWANTO</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>CZEXPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>80014155</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>HERI PRASETYO</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>GY1R12</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>80014095</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>HERMAWAN DWI SUPRIYADI</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>ZXRPUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>80017177</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
           <t>HOLLY AJI KUSUMA</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>S141RK</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>80009701</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>IRMAYADI</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>6JIT3C</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>80002118</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>JOHANSYAH</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>3314VX</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>80013827</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>KORINTUS DEPIN</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>G0SJGC</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>80017430</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>KORINTUS DEPIN</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>LCVLS4</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>80016612</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>LIANSYAH</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>9U9TLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>80004593</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>M ARJUNI</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>US26BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>80009577</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>MARDI ARYANTO</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>D5IRWX</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>80011723</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>MUHAMMAD MAHYUDDIN</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>0K3I52</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>80002120</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>MUHAMMAD SAID</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>PKXJQA</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>80009581</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>PARDIANSAH</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>CLOMD8</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>80008812</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>PENGKY ANGGARY</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>A0ZKHB</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>80017427</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>RESAL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>NZ844Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>80013760</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>RESAL</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>J87H3C</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>80008803</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>RINTO PARULIAN SITANGGANG</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>BG0KFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>80004079</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>RUSLI</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>WTANQT</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>80002253</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>SUPRIADI</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>7J6J78</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>80003010</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>TAUFIK HIDAYAT</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>9VGCO8</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>80016561</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>WAHYU</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>SI4FA5</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>80003140</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>WANDRA PRIMA PERA</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>A0CAWT</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>80009720</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>YASER ARAFAT</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>VU7UKL</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>80002654</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>YONATAN</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>NES171</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Force update dan amankan master Daftar_Akses_Portal.xlsx
</commit_message>
<xml_diff>
--- a/Daftar_Akses_Portal.xlsx
+++ b/Daftar_Akses_Portal.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,814 +441,2002 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>80002118</t>
+          <t>1611241</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>JOHANSYAH</t>
+          <t>AHMAD FADHOLI</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1QS2ZX</t>
+          <t>90P4OG</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>80001861</t>
+          <t>1508261</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AL FAIZAL WIJAYA</t>
+          <t>AHMAD FIRDAUS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>47GKTO</t>
+          <t>SW6HZF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>80002120</t>
+          <t>2006251</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MUHAMMAD SAID</t>
+          <t>AHMAD JURDI</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ZTOFYP</t>
+          <t>HS7IZ1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>80002253</t>
+          <t>1102261</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SUPRIADI</t>
+          <t>AHMAD KURNIAWAN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7EQ2ZP</t>
+          <t>JC6IIM</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>80003010</t>
+          <t>2804232</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TAUFIK HIDAYAT</t>
+          <t>AHMAD NOR</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>G25V2P</t>
+          <t>XY91YY</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>80003132</t>
+          <t>2802253</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BALINTON SITEPU</t>
+          <t>AHMAD YUNUS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CPO87C</t>
+          <t>MGIUWZ</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>80004079</t>
+          <t>207251</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RUSLI</t>
+          <t>AHMAT SUGIANOR</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IXRMYB</t>
+          <t>G8PA9F</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>80004296</t>
+          <t>2910241</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>HERI PORWANTO</t>
+          <t>ALDO WARTA SAPUTRA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2B0TA1</t>
+          <t>UMRSRH</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>80005321</t>
+          <t>206231</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>HENDRA GUNAWAN</t>
+          <t>AMANDA MARINDO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FAYC4X</t>
+          <t>9EV8PA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>80007180</t>
+          <t>201261</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>EKO NURYONO</t>
+          <t>AMINAL HUSNADI</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LRDC6H</t>
+          <t>9FYP9Q</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>80007834</t>
+          <t>200509251</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ABDUL  SALAM</t>
+          <t>ANDRE JEVISCA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LP1TSK</t>
+          <t>SASSNO</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>80008812</t>
+          <t>2405261</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PENGKY ANGGARY</t>
+          <t>BUDIMAN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2G1ZMV</t>
+          <t>A406YI</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>80009577</t>
+          <t>2405262</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MARDI ARYANTO</t>
+          <t>DAFRIT TIERO BERNANDO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>V1H5AE</t>
+          <t>JQY1FQ</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>80009581</t>
+          <t>202809251</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PARDIANSAH</t>
+          <t>DENIS DAMARA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>KYPHGF</t>
+          <t>KEYXNM</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>80009701</t>
+          <t>1706261</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>IRMAYADI</t>
+          <t>DWIKY RYAMIZARDIN</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>QHSYDL</t>
+          <t>RN7M9B</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>80013827</t>
+          <t>207231</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KORINTUS DEPIN</t>
+          <t>FAJAR PILIPUS SIHOMBING</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>VQ5ZOP</t>
+          <t>3JCPGE</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>80014093</t>
+          <t>1402231</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DANI DWI ADI RAHMADANA</t>
+          <t>HANSO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TS1B58</t>
+          <t>KSV76K</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>80014094</t>
+          <t>603222</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GATOT PRINGGO SUKOCO</t>
+          <t>IRFAN NURHADI</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C4FMAE</t>
+          <t>CP9801</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>80014095</t>
+          <t>2802252</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>HERMAWAN DWI SUPRIYADI</t>
+          <t>JIMI ARNOLDY</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>94VLZP</t>
+          <t>H5CHW9</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>80014153</t>
+          <t>1004253</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>FERY GUNAWAN</t>
+          <t>JUMILIN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>PFZFPX</t>
+          <t>A10EZK</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>80014154</t>
+          <t>200811251</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GIGIH SUTANTO</t>
+          <t>KOMOK</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>GJHGCX</t>
+          <t>R0P42T</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>80014155</t>
+          <t>1508264</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>HERI PRASETYO</t>
+          <t>LEWIS PRISTIANDI</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AXXM16</t>
+          <t>TVJ5FW</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>80017427</t>
+          <t>1004254</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>RESAL</t>
+          <t>LUTFY YAZID</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>H6ZZ9K</t>
+          <t>IQB46L</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>80017430</t>
+          <t>201409251</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>KORINTUS DEPIN</t>
+          <t>MILKANSYAH</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>7RNE9D</t>
+          <t>WLJVFK</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>80002654</t>
+          <t>1906253</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>YONATAN</t>
+          <t>MUHAMMAD AKHSANUL HUDA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>X1MS6D</t>
+          <t>P4A74O</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>80003140</t>
+          <t>1510243</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>WANDRA PRIMA PERA</t>
+          <t>MUHAMMAD HUSNI THAMRIN</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>8LK1QP</t>
+          <t>IJD3XQ</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>80004479</t>
+          <t>1912241</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GARANTO GURITNO</t>
+          <t>MUHAMMAD ISNUHONI</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5QJ4CI</t>
+          <t>BE3RP2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>80004593</t>
+          <t>1508262</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>M ARJUNI</t>
+          <t>MUHAMMAD REFFY FAHREZA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>I18QLD</t>
+          <t>DYKAZB</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>80006801</t>
+          <t>1508263</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AHMAD ANUGRAH MUFTI ALAM</t>
+          <t>MUHAMMAD RIDWAN</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>QA981W</t>
+          <t>7ATA8O</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>80008416</t>
+          <t>202809252</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AGUS</t>
+          <t>MUHAMMAD RIZKI FIRDAUS</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>8LP0XA</t>
+          <t>EC1A1C</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>80008803</t>
+          <t>2604251</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>RINTO PARULIAN SITANGGANG</t>
+          <t>MUHAMMAD ZAINI</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>RJRUTM</t>
+          <t>A3PMAE</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>80009720</t>
+          <t>1510241</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>YASER ARAFAT</t>
+          <t>NANDA RIZKY BUDIANTO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>QXLDEW</t>
+          <t>C4GZW9</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>80011723</t>
+          <t>2307261</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MUHAMMAD MAHYUDDIN</t>
+          <t>NOVARI FADLI</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>5OVE4Y</t>
+          <t>EZVF55</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>80013760</t>
+          <t>110241</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>RESAL</t>
+          <t>NOVITA FITRI</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>83CYVA</t>
+          <t>GZ2YYU</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>80016561</t>
+          <t>2703251</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>WAHYU</t>
+          <t>PIGAR</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>IJH1W8</t>
+          <t>OFA2G0</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>80016612</t>
+          <t>108235</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LIANSYAH</t>
+          <t>RANDI</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5BCXSN</t>
+          <t>JZXY70</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>NON STAFF</t>
+          <t>BMP</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>1705261</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>RESKI</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>NG9M5K</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1906252</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>REVALDHY NARADA PUTRA</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>9NGGZX</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>108238</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>RIFKY JANUARTA</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>S347C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>201409252</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ROSID WASKITO</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>E1KXOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1507261</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>SERBIANTO</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>BHCCOL</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1303221</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SUGIANOR</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>8YHR3Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2107261</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SYARIFUDIN</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>XBMWUX</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1004255</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>TEDY SAPUTRA</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>JZ3X61</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2103223</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>THANTAWI FADILAH</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>QDZD88</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>200509255</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>UKANDRI</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Q53JQK</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>207253</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>VRIO AGUSTINUS</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>WYRDHH</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2106234</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>WILDAN IRGIE FAZIRA</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>I39115</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BMP</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1906254</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ZAINAL HAKIM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>MQO5E0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>102111001</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>IZAH</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>6UENO5</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>202311002</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MADRI YANI</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>T85IQH</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>102311001</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>RISWANDI</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>JDR4DP</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>102401001</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>TAUFIK KURAHMAN</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>KLV1JT</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CMU</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>10151021</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>YOKO</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>040G2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>80007834</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ABDUL  SALAM</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>LP1TSK</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>80008416</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>AGUS</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>8LP0XA</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>80006801</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>AHMAD ANUGRAH MUFTI ALAM</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>QA981W</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>80001861</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>AL FAIZAL WIJAYA</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>47GKTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>80003132</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>BALINTON SITEPU</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>CPO87C</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>80014093</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>DANI DWI ADI RAHMADANA</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TS1B58</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>80007180</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>EKO NURYONO</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>LRDC6H</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>80014153</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>FERY GUNAWAN</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>PFZFPX</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>80004479</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>GARANTO GURITNO</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>5QJ4CI</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>80014094</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>GATOT PRINGGO SUKOCO</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>C4FMAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>80014154</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>GIGIH SUTANTO</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>GJHGCX</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>80005321</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>HENDRA GUNAWAN</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>FAYC4X</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>80004296</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>HERI PORWANTO</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>2B0TA1</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>80014155</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>HERI PRASETYO</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>AXXM16</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>80014095</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>HERMAWAN DWI SUPRIYADI</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>94VLZP</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
           <t>80017177</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>HOLLY AJI KUSUMA</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>B3WPZV</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>80009701</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>IRMAYADI</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>QHSYDL</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>80002118</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>JOHANSYAH</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>1QS2ZX</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>80013827</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>KORINTUS DEPIN</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>VQ5ZOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>80017430</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>KORINTUS DEPIN</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>7RNE9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>80016612</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>LIANSYAH</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>5BCXSN</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>80004593</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>M ARJUNI</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>I18QLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>80009577</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>MARDI ARYANTO</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>V1H5AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>80011723</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>MUHAMMAD MAHYUDDIN</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>5OVE4Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>80002120</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>MUHAMMAD SAID</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>ZTOFYP</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>80009581</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>PARDIANSAH</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>KYPHGF</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>80008812</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>PENGKY ANGGARY</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>2G1ZMV</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>80017427</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>RESAL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>H6ZZ9K</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>80013760</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>RESAL</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>83CYVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>80008803</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>RINTO PARULIAN SITANGGANG</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>RJRUTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>80004079</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>RUSLI</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>IXRMYB</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>80002253</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>SUPRIADI</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>7EQ2ZP</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>80003010</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>TAUFIK HIDAYAT</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>G25V2P</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>80016561</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>WAHYU</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>IJH1W8</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>80003140</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>WANDRA PRIMA PERA</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>8LK1QP</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>80009720</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>YASER ARAFAT</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>QXLDEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>NON STAFF</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>80002654</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>YONATAN</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>X1MS6D</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
mengubah tampilan login dan dashboard
</commit_message>
<xml_diff>
--- a/Daftar_Akses_Portal.xlsx
+++ b/Daftar_Akses_Portal.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GENERAL PSD\PENDINGAN LINDAA 2026\GENERAL 2026\00. PORTAL TIMESHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26785630-F98C-460F-A1A6-BA62BD2A4596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{587FAF72-C008-40C2-94A6-060D83627A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="270">
   <si>
     <t>Perusahaan</t>
   </si>
@@ -280,18 +293,12 @@
     <t>BE3RP2</t>
   </si>
   <si>
-    <t>1508262</t>
-  </si>
-  <si>
     <t>MUHAMMAD REFFY FAHREZA</t>
   </si>
   <si>
     <t>DYKAZB</t>
   </si>
   <si>
-    <t>1508263</t>
-  </si>
-  <si>
     <t>MUHAMMAD RIDWAN</t>
   </si>
   <si>
@@ -433,9 +440,6 @@
     <t>JZ3X61</t>
   </si>
   <si>
-    <t>2103223</t>
-  </si>
-  <si>
     <t>THANTAWI FADILAH</t>
   </si>
   <si>
@@ -499,9 +503,6 @@
     <t>T85IQH</t>
   </si>
   <si>
-    <t>102311001</t>
-  </si>
-  <si>
     <t>RISWANDI</t>
   </si>
   <si>
@@ -517,9 +518,6 @@
     <t>KLV1JT</t>
   </si>
   <si>
-    <t>10151021</t>
-  </si>
-  <si>
     <t>YOKO</t>
   </si>
   <si>
@@ -529,9 +527,6 @@
     <t>NON STAFF</t>
   </si>
   <si>
-    <t>80007834</t>
-  </si>
-  <si>
     <t>ABDUL  SALAM</t>
   </si>
   <si>
@@ -572,9 +567,6 @@
   </si>
   <si>
     <t>CPO87C</t>
-  </si>
-  <si>
-    <t>80014093</t>
   </si>
   <si>
     <t>DANI DWI ADI RAHMADANA</t>
@@ -886,8 +878,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1193,6 +1188,7 @@
   <dimension ref="A1:D92"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1593,28 +1589,28 @@
       <c r="A29" t="s">
         <v>4</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29">
+        <v>1508262</v>
+      </c>
+      <c r="C29" t="s">
         <v>86</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>87</v>
-      </c>
-      <c r="D29" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>4</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30">
+        <v>1508263</v>
+      </c>
+      <c r="C30" t="s">
+        <v>88</v>
+      </c>
+      <c r="D30" t="s">
         <v>89</v>
-      </c>
-      <c r="C30" t="s">
-        <v>90</v>
-      </c>
-      <c r="D30" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
@@ -1622,13 +1618,13 @@
         <v>4</v>
       </c>
       <c r="B31" t="s">
+        <v>90</v>
+      </c>
+      <c r="C31" t="s">
+        <v>91</v>
+      </c>
+      <c r="D31" t="s">
         <v>92</v>
-      </c>
-      <c r="C31" t="s">
-        <v>93</v>
-      </c>
-      <c r="D31" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
@@ -1636,13 +1632,13 @@
         <v>4</v>
       </c>
       <c r="B32" t="s">
+        <v>93</v>
+      </c>
+      <c r="C32" t="s">
+        <v>94</v>
+      </c>
+      <c r="D32" t="s">
         <v>95</v>
-      </c>
-      <c r="C32" t="s">
-        <v>96</v>
-      </c>
-      <c r="D32" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -1650,13 +1646,13 @@
         <v>4</v>
       </c>
       <c r="B33" t="s">
+        <v>96</v>
+      </c>
+      <c r="C33" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" t="s">
         <v>98</v>
-      </c>
-      <c r="C33" t="s">
-        <v>99</v>
-      </c>
-      <c r="D33" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
@@ -1664,13 +1660,13 @@
         <v>4</v>
       </c>
       <c r="B34" t="s">
+        <v>99</v>
+      </c>
+      <c r="C34" t="s">
+        <v>100</v>
+      </c>
+      <c r="D34" t="s">
         <v>101</v>
-      </c>
-      <c r="C34" t="s">
-        <v>102</v>
-      </c>
-      <c r="D34" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -1678,13 +1674,13 @@
         <v>4</v>
       </c>
       <c r="B35" t="s">
+        <v>102</v>
+      </c>
+      <c r="C35" t="s">
+        <v>103</v>
+      </c>
+      <c r="D35" t="s">
         <v>104</v>
-      </c>
-      <c r="C35" t="s">
-        <v>105</v>
-      </c>
-      <c r="D35" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -1692,13 +1688,13 @@
         <v>4</v>
       </c>
       <c r="B36" t="s">
+        <v>105</v>
+      </c>
+      <c r="C36" t="s">
+        <v>106</v>
+      </c>
+      <c r="D36" t="s">
         <v>107</v>
-      </c>
-      <c r="C36" t="s">
-        <v>108</v>
-      </c>
-      <c r="D36" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
@@ -1706,13 +1702,13 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" t="s">
+        <v>109</v>
+      </c>
+      <c r="D37" t="s">
         <v>110</v>
-      </c>
-      <c r="C37" t="s">
-        <v>111</v>
-      </c>
-      <c r="D37" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -1720,13 +1716,13 @@
         <v>4</v>
       </c>
       <c r="B38" t="s">
+        <v>111</v>
+      </c>
+      <c r="C38" t="s">
+        <v>112</v>
+      </c>
+      <c r="D38" t="s">
         <v>113</v>
-      </c>
-      <c r="C38" t="s">
-        <v>114</v>
-      </c>
-      <c r="D38" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -1734,13 +1730,13 @@
         <v>4</v>
       </c>
       <c r="B39" t="s">
+        <v>114</v>
+      </c>
+      <c r="C39" t="s">
+        <v>115</v>
+      </c>
+      <c r="D39" t="s">
         <v>116</v>
-      </c>
-      <c r="C39" t="s">
-        <v>117</v>
-      </c>
-      <c r="D39" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
@@ -1748,13 +1744,13 @@
         <v>4</v>
       </c>
       <c r="B40" t="s">
+        <v>117</v>
+      </c>
+      <c r="C40" t="s">
+        <v>118</v>
+      </c>
+      <c r="D40" t="s">
         <v>119</v>
-      </c>
-      <c r="C40" t="s">
-        <v>120</v>
-      </c>
-      <c r="D40" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
@@ -1762,13 +1758,13 @@
         <v>4</v>
       </c>
       <c r="B41" t="s">
+        <v>120</v>
+      </c>
+      <c r="C41" t="s">
+        <v>121</v>
+      </c>
+      <c r="D41" t="s">
         <v>122</v>
-      </c>
-      <c r="C41" t="s">
-        <v>123</v>
-      </c>
-      <c r="D41" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
@@ -1776,13 +1772,13 @@
         <v>4</v>
       </c>
       <c r="B42" t="s">
+        <v>123</v>
+      </c>
+      <c r="C42" t="s">
+        <v>124</v>
+      </c>
+      <c r="D42" t="s">
         <v>125</v>
-      </c>
-      <c r="C42" t="s">
-        <v>126</v>
-      </c>
-      <c r="D42" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -1790,699 +1786,699 @@
         <v>4</v>
       </c>
       <c r="B43" t="s">
+        <v>126</v>
+      </c>
+      <c r="C43" t="s">
+        <v>127</v>
+      </c>
+      <c r="D43" t="s">
         <v>128</v>
-      </c>
-      <c r="C43" t="s">
-        <v>129</v>
-      </c>
-      <c r="D43" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>4</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C44" t="s">
+        <v>130</v>
+      </c>
+      <c r="D44" t="s">
         <v>131</v>
-      </c>
-      <c r="C44" t="s">
-        <v>132</v>
-      </c>
-      <c r="D44" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>4</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C45" t="s">
+        <v>133</v>
+      </c>
+      <c r="D45" t="s">
         <v>134</v>
-      </c>
-      <c r="C45" t="s">
-        <v>135</v>
-      </c>
-      <c r="D45" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>4</v>
       </c>
-      <c r="B46" t="s">
-        <v>137</v>
+      <c r="B46" s="1">
+        <v>2103223</v>
       </c>
       <c r="C46" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D46" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>4</v>
       </c>
-      <c r="B47" t="s">
-        <v>140</v>
+      <c r="B47" s="1" t="s">
+        <v>137</v>
       </c>
       <c r="C47" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D47" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>4</v>
       </c>
-      <c r="B48" t="s">
-        <v>143</v>
+      <c r="B48" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="C48" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D48" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>4</v>
       </c>
-      <c r="B49" t="s">
-        <v>146</v>
+      <c r="B49" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="C49" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D49" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>4</v>
       </c>
-      <c r="B50" t="s">
-        <v>149</v>
+      <c r="B50" s="1" t="s">
+        <v>146</v>
       </c>
       <c r="C50" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D50" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
+        <v>149</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C51" t="s">
+        <v>151</v>
+      </c>
+      <c r="D51" t="s">
         <v>152</v>
-      </c>
-      <c r="B51" t="s">
-        <v>153</v>
-      </c>
-      <c r="C51" t="s">
-        <v>154</v>
-      </c>
-      <c r="D51" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>152</v>
-      </c>
-      <c r="B52" t="s">
-        <v>156</v>
+        <v>149</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>153</v>
       </c>
       <c r="C52" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D52" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>152</v>
-      </c>
-      <c r="B53" t="s">
-        <v>159</v>
+        <v>149</v>
+      </c>
+      <c r="B53" s="1">
+        <v>102311001</v>
       </c>
       <c r="C53" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D53" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>152</v>
-      </c>
-      <c r="B54" t="s">
-        <v>162</v>
+        <v>149</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>158</v>
       </c>
       <c r="C54" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D54" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>152</v>
-      </c>
-      <c r="B55" t="s">
-        <v>165</v>
+        <v>149</v>
+      </c>
+      <c r="B55" s="1">
+        <v>10151021</v>
       </c>
       <c r="C55" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D55" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>168</v>
-      </c>
-      <c r="B56" t="s">
-        <v>169</v>
+        <v>163</v>
+      </c>
+      <c r="B56" s="1">
+        <v>80007834</v>
       </c>
       <c r="C56" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="D56" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
+        <v>163</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C57" t="s">
+        <v>167</v>
+      </c>
+      <c r="D57" t="s">
         <v>168</v>
-      </c>
-      <c r="B57" t="s">
-        <v>172</v>
-      </c>
-      <c r="C57" t="s">
-        <v>173</v>
-      </c>
-      <c r="D57" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>168</v>
-      </c>
-      <c r="B58" t="s">
-        <v>175</v>
+        <v>163</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>169</v>
       </c>
       <c r="C58" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D58" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>168</v>
-      </c>
-      <c r="B59" t="s">
-        <v>178</v>
+        <v>163</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>172</v>
       </c>
       <c r="C59" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D59" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>168</v>
-      </c>
-      <c r="B60" t="s">
-        <v>181</v>
+        <v>163</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>175</v>
       </c>
       <c r="C60" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D60" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>168</v>
-      </c>
-      <c r="B61" t="s">
-        <v>184</v>
+        <v>163</v>
+      </c>
+      <c r="B61" s="1">
+        <v>80014093</v>
       </c>
       <c r="C61" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D61" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>168</v>
-      </c>
-      <c r="B62" t="s">
-        <v>187</v>
+        <v>163</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>180</v>
       </c>
       <c r="C62" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="D62" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>168</v>
-      </c>
-      <c r="B63" t="s">
-        <v>190</v>
+        <v>163</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>183</v>
       </c>
       <c r="C63" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="D63" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>168</v>
-      </c>
-      <c r="B64">
+        <v>163</v>
+      </c>
+      <c r="B64" s="1">
         <v>80004479</v>
       </c>
       <c r="C64" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D64" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>168</v>
-      </c>
-      <c r="B65" t="s">
-        <v>195</v>
+        <v>163</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>188</v>
       </c>
       <c r="C65" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="D65" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>168</v>
-      </c>
-      <c r="B66" t="s">
-        <v>198</v>
+        <v>163</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>191</v>
       </c>
       <c r="C66" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="D66" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>168</v>
-      </c>
-      <c r="B67" t="s">
-        <v>201</v>
+        <v>163</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>194</v>
       </c>
       <c r="C67" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="D67" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>168</v>
-      </c>
-      <c r="B68" t="s">
-        <v>204</v>
+        <v>163</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>197</v>
       </c>
       <c r="C68" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="D68" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>168</v>
-      </c>
-      <c r="B69" t="s">
-        <v>207</v>
+        <v>163</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>200</v>
       </c>
       <c r="C69" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D69" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B70" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C70" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="D70" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B71" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="C71" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="D71" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B72" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="C72" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="D72" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B73" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="C73" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="D73" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B74" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="C74" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="D74" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B75" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="C75" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="D75" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B76" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="C76" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="D76" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B77" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="C77" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="D77" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B78" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="C78" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="D78" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B79" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C79" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="D79" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B80" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C80" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D80" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B81" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C81" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="D81" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B82" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="C82" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="D82" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B83" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C83" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="D83" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B84" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C84" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="D84" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B85" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="C85" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="D85" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B86" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="C86" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="D86" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B87" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="C87" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="D87" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B88" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="C88" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="D88" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B89" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="C89" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="D89" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B90" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="C90" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="D90" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B91" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="C91" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="D91" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B92" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="C92" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="D92" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
revisi ulang tampilan dashboard
</commit_message>
<xml_diff>
--- a/Daftar_Akses_Portal.xlsx
+++ b/Daftar_Akses_Portal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GENERAL PSD\PENDINGAN LINDAA 2026\GENERAL 2026\00. PORTAL TIMESHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{587FAF72-C008-40C2-94A6-060D83627A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1421A4-F95C-462A-9FC5-2FFA8C3FE5E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="267">
   <si>
     <t>Perusahaan</t>
   </si>
@@ -50,9 +50,6 @@
     <t>BMP</t>
   </si>
   <si>
-    <t>1611241</t>
-  </si>
-  <si>
     <t>AHMAD FADHOLI</t>
   </si>
   <si>
@@ -140,16 +137,10 @@
     <t>9FYP9Q</t>
   </si>
   <si>
-    <t>200509251</t>
-  </si>
-  <si>
     <t>ANDRE JEVISCA</t>
   </si>
   <si>
     <t>SASSNO</t>
-  </si>
-  <si>
-    <t>2405261</t>
   </si>
   <si>
     <t>BUDIMAN</t>
@@ -1211,14 +1202,14 @@
       <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2">
+        <v>1611241</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1226,13 +1217,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1240,13 +1231,13 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -1254,13 +1245,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>15</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -1268,13 +1259,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>18</v>
-      </c>
-      <c r="D6" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -1282,13 +1273,13 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -1296,13 +1287,13 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
         <v>23</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>24</v>
-      </c>
-      <c r="D8" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -1310,13 +1301,13 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
         <v>26</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>27</v>
-      </c>
-      <c r="D9" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -1324,13 +1315,13 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
         <v>29</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>30</v>
-      </c>
-      <c r="D10" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -1338,41 +1329,41 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
         <v>32</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>33</v>
-      </c>
-      <c r="D11" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>4</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12">
+        <v>200509251</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" t="s">
         <v>35</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>4</v>
       </c>
-      <c r="B13" t="s">
-        <v>38</v>
+      <c r="B13">
+        <v>2405261</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -1380,13 +1371,13 @@
         <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D14" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -1394,13 +1385,13 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
@@ -1408,13 +1399,13 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
@@ -1422,13 +1413,13 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -1436,13 +1427,13 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D18" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -1450,13 +1441,13 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -1464,13 +1455,13 @@
         <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C20" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D20" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -1478,13 +1469,13 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D21" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -1492,13 +1483,13 @@
         <v>4</v>
       </c>
       <c r="B22" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C22" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -1506,13 +1497,13 @@
         <v>4</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C23" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D23" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -1520,13 +1511,13 @@
         <v>4</v>
       </c>
       <c r="B24" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C24" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D24" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -1534,13 +1525,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C25" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D25" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -1548,13 +1539,13 @@
         <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C26" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D26" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -1562,13 +1553,13 @@
         <v>4</v>
       </c>
       <c r="B27" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C27" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D27" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
@@ -1576,13 +1567,13 @@
         <v>4</v>
       </c>
       <c r="B28" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C28" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D28" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -1593,10 +1584,10 @@
         <v>1508262</v>
       </c>
       <c r="C29" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D29" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
@@ -1607,10 +1598,10 @@
         <v>1508263</v>
       </c>
       <c r="C30" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D30" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
@@ -1618,13 +1609,13 @@
         <v>4</v>
       </c>
       <c r="B31" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C31" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D31" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
@@ -1632,13 +1623,13 @@
         <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C32" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D32" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -1646,13 +1637,13 @@
         <v>4</v>
       </c>
       <c r="B33" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C33" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D33" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
@@ -1660,13 +1651,13 @@
         <v>4</v>
       </c>
       <c r="B34" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C34" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D34" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -1674,13 +1665,13 @@
         <v>4</v>
       </c>
       <c r="B35" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C35" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D35" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -1688,13 +1679,13 @@
         <v>4</v>
       </c>
       <c r="B36" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C36" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D36" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
@@ -1702,13 +1693,13 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C37" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D37" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -1716,13 +1707,13 @@
         <v>4</v>
       </c>
       <c r="B38" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C38" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D38" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -1730,13 +1721,13 @@
         <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C39" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D39" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
@@ -1744,13 +1735,13 @@
         <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C40" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D40" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
@@ -1758,13 +1749,13 @@
         <v>4</v>
       </c>
       <c r="B41" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C41" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D41" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
@@ -1772,13 +1763,13 @@
         <v>4</v>
       </c>
       <c r="B42" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C42" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D42" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -1786,13 +1777,13 @@
         <v>4</v>
       </c>
       <c r="B43" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C43" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D43" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
@@ -1800,13 +1791,13 @@
         <v>4</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C44" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D44" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
@@ -1814,13 +1805,13 @@
         <v>4</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C45" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D45" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
@@ -1831,10 +1822,10 @@
         <v>2103223</v>
       </c>
       <c r="C46" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D46" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
@@ -1842,13 +1833,13 @@
         <v>4</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D47" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
@@ -1856,13 +1847,13 @@
         <v>4</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C48" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D48" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
@@ -1870,13 +1861,13 @@
         <v>4</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C49" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D49" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
@@ -1884,601 +1875,601 @@
         <v>4</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C50" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D50" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
+        <v>146</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C51" t="s">
+        <v>148</v>
+      </c>
+      <c r="D51" t="s">
         <v>149</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="C51" t="s">
-        <v>151</v>
-      </c>
-      <c r="D51" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C52" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D52" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B53" s="1">
         <v>102311001</v>
       </c>
       <c r="C53" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D53" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C54" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D54" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B55" s="1">
         <v>10151021</v>
       </c>
       <c r="C55" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D55" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B56" s="1">
         <v>80007834</v>
       </c>
       <c r="C56" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D56" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
+        <v>160</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B57" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="C57" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D57" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C58" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D58" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C59" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D59" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C60" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D60" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B61" s="1">
         <v>80014093</v>
       </c>
       <c r="C61" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D61" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C62" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D62" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C63" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D63" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B64" s="1">
         <v>80004479</v>
       </c>
       <c r="C64" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D64" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C65" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D65" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C66" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D66" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C67" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D67" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C68" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D68" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C69" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D69" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B70" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C70" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D70" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B71" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C71" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D71" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B72" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C72" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D72" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B73" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C73" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D73" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B74" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C74" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D74" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B75" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C75" t="s">
+        <v>213</v>
+      </c>
+      <c r="D75" t="s">
         <v>216</v>
-      </c>
-      <c r="D75" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B76" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C76" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D76" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B77" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C77" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D77" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B78" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C78" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D78" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B79" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C79" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D79" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B80" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C80" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D80" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B81" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C81" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D81" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B82" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C82" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D82" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B83" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C83" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D83" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B84" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C84" t="s">
+        <v>239</v>
+      </c>
+      <c r="D84" t="s">
         <v>242</v>
-      </c>
-      <c r="D84" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B85" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C85" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D85" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B86" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="C86" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D86" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B87" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C87" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D87" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B88" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C88" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D88" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B89" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C89" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D89" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B90" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C90" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D90" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B91" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C91" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D91" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B92" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C92" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D92" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update admin portal dan struktur folder
</commit_message>
<xml_diff>
--- a/Daftar_Akses_Portal.xlsx
+++ b/Daftar_Akses_Portal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GENERAL PSD\PENDINGAN LINDAA 2026\GENERAL 2026\00. PORTAL TIMESHEET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1421A4-F95C-462A-9FC5-2FFA8C3FE5E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7C23D36-727E-4F0B-880B-D31EACAAA218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="249">
   <si>
     <t>Perusahaan</t>
   </si>
@@ -56,81 +56,54 @@
     <t>90P4OG</t>
   </si>
   <si>
-    <t>1508261</t>
-  </si>
-  <si>
     <t>AHMAD FIRDAUS</t>
   </si>
   <si>
     <t>SW6HZF</t>
   </si>
   <si>
-    <t>2006251</t>
-  </si>
-  <si>
     <t>AHMAD JURDI</t>
   </si>
   <si>
     <t>HS7IZ1</t>
   </si>
   <si>
-    <t>1102261</t>
-  </si>
-  <si>
     <t>AHMAD KURNIAWAN</t>
   </si>
   <si>
     <t>JC6IIM</t>
   </si>
   <si>
-    <t>2804232</t>
-  </si>
-  <si>
     <t>AHMAD NOR</t>
   </si>
   <si>
     <t>XY91YY</t>
   </si>
   <si>
-    <t>2802253</t>
-  </si>
-  <si>
     <t>AHMAD YUNUS</t>
   </si>
   <si>
     <t>MGIUWZ</t>
   </si>
   <si>
-    <t>207251</t>
-  </si>
-  <si>
     <t>AHMAT SUGIANOR</t>
   </si>
   <si>
     <t>G8PA9F</t>
   </si>
   <si>
-    <t>2910241</t>
-  </si>
-  <si>
     <t>ALDO WARTA SAPUTRA</t>
   </si>
   <si>
     <t>UMRSRH</t>
   </si>
   <si>
-    <t>206231</t>
-  </si>
-  <si>
     <t>AMANDA MARINDO</t>
   </si>
   <si>
     <t>9EV8PA</t>
   </si>
   <si>
-    <t>201261</t>
-  </si>
-  <si>
     <t>AMINAL HUSNADI</t>
   </si>
   <si>
@@ -149,36 +122,24 @@
     <t>A406YI</t>
   </si>
   <si>
-    <t>2405262</t>
-  </si>
-  <si>
     <t>DAFRIT TIERO BERNANDO</t>
   </si>
   <si>
     <t>JQY1FQ</t>
   </si>
   <si>
-    <t>202809251</t>
-  </si>
-  <si>
     <t>DENIS DAMARA</t>
   </si>
   <si>
     <t>KEYXNM</t>
   </si>
   <si>
-    <t>1706261</t>
-  </si>
-  <si>
     <t>DWIKY RYAMIZARDIN</t>
   </si>
   <si>
     <t>RN7M9B</t>
   </si>
   <si>
-    <t>207231</t>
-  </si>
-  <si>
     <t>FAJAR PILIPUS SIHOMBING</t>
   </si>
   <si>
@@ -476,18 +437,12 @@
     <t>CMU</t>
   </si>
   <si>
-    <t>102111001</t>
-  </si>
-  <si>
     <t>IZAH</t>
   </si>
   <si>
     <t>6UENO5</t>
   </si>
   <si>
-    <t>202311002</t>
-  </si>
-  <si>
     <t>MADRI YANI</t>
   </si>
   <si>
@@ -500,9 +455,6 @@
     <t>JDR4DP</t>
   </si>
   <si>
-    <t>102401001</t>
-  </si>
-  <si>
     <t>TAUFIK KURAHMAN</t>
   </si>
   <si>
@@ -524,9 +476,6 @@
     <t>LP1TSK</t>
   </si>
   <si>
-    <t>80008416</t>
-  </si>
-  <si>
     <t>AGUS</t>
   </si>
   <si>
@@ -540,9 +489,6 @@
   </si>
   <si>
     <t>QA981W</t>
-  </si>
-  <si>
-    <t>80001861</t>
   </si>
   <si>
     <t>AL FAIZAL WIJAYA</t>
@@ -1216,126 +1162,126 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3">
+        <v>1508261</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4">
+        <v>2006251</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
         <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>13</v>
+      <c r="B5">
+        <v>1102261</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
-        <v>16</v>
+      <c r="B6">
+        <v>2804232</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>4</v>
       </c>
-      <c r="B7" t="s">
-        <v>19</v>
+      <c r="B7">
+        <v>2802253</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>4</v>
       </c>
-      <c r="B8" t="s">
-        <v>22</v>
+      <c r="B8">
+        <v>207251</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>4</v>
       </c>
-      <c r="B9" t="s">
-        <v>25</v>
+      <c r="B9">
+        <v>2910241</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>4</v>
       </c>
-      <c r="B10" t="s">
-        <v>28</v>
+      <c r="B10">
+        <v>206231</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>4</v>
       </c>
-      <c r="B11" t="s">
-        <v>31</v>
+      <c r="B11">
+        <v>201261</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -1346,10 +1292,10 @@
         <v>200509251</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -1360,66 +1306,66 @@
         <v>2405261</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>4</v>
       </c>
-      <c r="B14" t="s">
-        <v>38</v>
+      <c r="B14">
+        <v>2405262</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>4</v>
       </c>
-      <c r="B15" t="s">
-        <v>41</v>
+      <c r="B15">
+        <v>202809251</v>
       </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="D15" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>4</v>
       </c>
-      <c r="B16" t="s">
-        <v>44</v>
+      <c r="B16">
+        <v>1706261</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>4</v>
       </c>
-      <c r="B17" t="s">
-        <v>47</v>
+      <c r="B17">
+        <v>207231</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -1427,13 +1373,13 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -1441,13 +1387,13 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="D19" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -1455,13 +1401,13 @@
         <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="D20" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -1469,13 +1415,13 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="D21" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -1483,13 +1429,13 @@
         <v>4</v>
       </c>
       <c r="B22" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="D22" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -1497,13 +1443,13 @@
         <v>4</v>
       </c>
       <c r="B23" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="C23" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="D23" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -1511,13 +1457,13 @@
         <v>4</v>
       </c>
       <c r="B24" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="D24" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -1525,13 +1471,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="D25" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -1539,13 +1485,13 @@
         <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="C26" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="D26" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -1553,13 +1499,13 @@
         <v>4</v>
       </c>
       <c r="B27" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C27" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
@@ -1567,13 +1513,13 @@
         <v>4</v>
       </c>
       <c r="B28" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="C28" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="D28" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -1584,10 +1530,10 @@
         <v>1508262</v>
       </c>
       <c r="C29" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="D29" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
@@ -1598,10 +1544,10 @@
         <v>1508263</v>
       </c>
       <c r="C30" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="D30" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
@@ -1609,13 +1555,13 @@
         <v>4</v>
       </c>
       <c r="B31" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="C31" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D31" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
@@ -1623,13 +1569,13 @@
         <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="C32" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="D32" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
@@ -1637,13 +1583,13 @@
         <v>4</v>
       </c>
       <c r="B33" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="C33" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="D33" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
@@ -1651,13 +1597,13 @@
         <v>4</v>
       </c>
       <c r="B34" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="C34" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="D34" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
@@ -1665,13 +1611,13 @@
         <v>4</v>
       </c>
       <c r="B35" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="C35" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="D35" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
@@ -1679,13 +1625,13 @@
         <v>4</v>
       </c>
       <c r="B36" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="C36" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="D36" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
@@ -1693,13 +1639,13 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="C37" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="D37" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
@@ -1707,13 +1653,13 @@
         <v>4</v>
       </c>
       <c r="B38" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C38" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="D38" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
@@ -1721,13 +1667,13 @@
         <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="C39" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="D39" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
@@ -1735,13 +1681,13 @@
         <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="C40" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="D40" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
@@ -1749,13 +1695,13 @@
         <v>4</v>
       </c>
       <c r="B41" t="s">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="C41" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="D41" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
@@ -1763,13 +1709,13 @@
         <v>4</v>
       </c>
       <c r="B42" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="C42" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="D42" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -1777,13 +1723,13 @@
         <v>4</v>
       </c>
       <c r="B43" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="C43" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="D43" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
@@ -1791,13 +1737,13 @@
         <v>4</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="C44" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="D44" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
@@ -1805,13 +1751,13 @@
         <v>4</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="C45" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="D45" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
@@ -1822,10 +1768,10 @@
         <v>2103223</v>
       </c>
       <c r="C46" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="D46" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
@@ -1833,13 +1779,13 @@
         <v>4</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="C47" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="D47" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
@@ -1847,13 +1793,13 @@
         <v>4</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="C48" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="D48" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
@@ -1861,13 +1807,13 @@
         <v>4</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="C49" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="D49" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
@@ -1875,601 +1821,601 @@
         <v>4</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="C50" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="D50" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>146</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>147</v>
+        <v>133</v>
+      </c>
+      <c r="B51" s="1">
+        <v>102111001</v>
       </c>
       <c r="C51" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="D51" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>146</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>150</v>
+        <v>133</v>
+      </c>
+      <c r="B52" s="1">
+        <v>202311002</v>
       </c>
       <c r="C52" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="D52" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="B53" s="1">
         <v>102311001</v>
       </c>
       <c r="C53" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="D53" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>146</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>155</v>
+        <v>133</v>
+      </c>
+      <c r="B54" s="1">
+        <v>102401001</v>
       </c>
       <c r="C54" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="D54" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="B55" s="1">
         <v>10151021</v>
       </c>
       <c r="C55" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="D55" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B56" s="1">
         <v>80007834</v>
       </c>
       <c r="C56" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="D56" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>160</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>163</v>
+        <v>144</v>
+      </c>
+      <c r="B57" s="1">
+        <v>80008416</v>
       </c>
       <c r="C57" t="s">
-        <v>164</v>
+        <v>147</v>
       </c>
       <c r="D57" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
       <c r="C58" t="s">
-        <v>167</v>
+        <v>150</v>
       </c>
       <c r="D58" t="s">
-        <v>168</v>
+        <v>151</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>160</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>169</v>
+        <v>144</v>
+      </c>
+      <c r="B59" s="1">
+        <v>80001861</v>
       </c>
       <c r="C59" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="D59" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="C60" t="s">
-        <v>173</v>
+        <v>155</v>
       </c>
       <c r="D60" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B61" s="1">
         <v>80014093</v>
       </c>
       <c r="C61" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="D61" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
+        <v>144</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C62" t="s">
         <v>160</v>
       </c>
-      <c r="B62" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="C62" t="s">
-        <v>178</v>
-      </c>
       <c r="D62" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="C63" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="D63" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B64" s="1">
         <v>80004479</v>
       </c>
       <c r="C64" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="D64" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="C65" t="s">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="D65" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="C66" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="D66" t="s">
-        <v>190</v>
+        <v>172</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>191</v>
+        <v>173</v>
       </c>
       <c r="C67" t="s">
-        <v>192</v>
+        <v>174</v>
       </c>
       <c r="D67" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="C68" t="s">
-        <v>195</v>
+        <v>177</v>
       </c>
       <c r="D68" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="C69" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="D69" t="s">
-        <v>199</v>
+        <v>181</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B70" t="s">
-        <v>200</v>
+        <v>182</v>
       </c>
       <c r="C70" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="D70" t="s">
-        <v>202</v>
+        <v>184</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B71" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="C71" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="D71" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B72" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="C72" t="s">
-        <v>207</v>
+        <v>189</v>
       </c>
       <c r="D72" t="s">
-        <v>208</v>
+        <v>190</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B73" t="s">
-        <v>209</v>
+        <v>191</v>
       </c>
       <c r="C73" t="s">
-        <v>210</v>
+        <v>192</v>
       </c>
       <c r="D73" t="s">
-        <v>211</v>
+        <v>193</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B74" t="s">
-        <v>212</v>
+        <v>194</v>
       </c>
       <c r="C74" t="s">
-        <v>213</v>
+        <v>195</v>
       </c>
       <c r="D74" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B75" t="s">
-        <v>215</v>
+        <v>197</v>
       </c>
       <c r="C75" t="s">
-        <v>213</v>
+        <v>195</v>
       </c>
       <c r="D75" t="s">
-        <v>216</v>
+        <v>198</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B76" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
       <c r="C76" t="s">
-        <v>218</v>
+        <v>200</v>
       </c>
       <c r="D76" t="s">
-        <v>219</v>
+        <v>201</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B77" t="s">
-        <v>220</v>
+        <v>202</v>
       </c>
       <c r="C77" t="s">
-        <v>221</v>
+        <v>203</v>
       </c>
       <c r="D77" t="s">
-        <v>222</v>
+        <v>204</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B78" t="s">
-        <v>223</v>
+        <v>205</v>
       </c>
       <c r="C78" t="s">
-        <v>224</v>
+        <v>206</v>
       </c>
       <c r="D78" t="s">
-        <v>225</v>
+        <v>207</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B79" t="s">
-        <v>226</v>
+        <v>208</v>
       </c>
       <c r="C79" t="s">
-        <v>227</v>
+        <v>209</v>
       </c>
       <c r="D79" t="s">
-        <v>228</v>
+        <v>210</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B80" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="C80" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="D80" t="s">
-        <v>231</v>
+        <v>213</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B81" t="s">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="C81" t="s">
-        <v>233</v>
+        <v>215</v>
       </c>
       <c r="D81" t="s">
-        <v>234</v>
+        <v>216</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B82" t="s">
-        <v>235</v>
+        <v>217</v>
       </c>
       <c r="C82" t="s">
-        <v>236</v>
+        <v>218</v>
       </c>
       <c r="D82" t="s">
-        <v>237</v>
+        <v>219</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B83" t="s">
-        <v>238</v>
+        <v>220</v>
       </c>
       <c r="C83" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="D83" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B84" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="C84" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="D84" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B85" t="s">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="C85" t="s">
-        <v>244</v>
+        <v>226</v>
       </c>
       <c r="D85" t="s">
-        <v>245</v>
+        <v>227</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B86" t="s">
-        <v>246</v>
+        <v>228</v>
       </c>
       <c r="C86" t="s">
-        <v>247</v>
+        <v>229</v>
       </c>
       <c r="D86" t="s">
-        <v>248</v>
+        <v>230</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B87" t="s">
-        <v>249</v>
+        <v>231</v>
       </c>
       <c r="C87" t="s">
-        <v>250</v>
+        <v>232</v>
       </c>
       <c r="D87" t="s">
-        <v>251</v>
+        <v>233</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B88" t="s">
-        <v>252</v>
+        <v>234</v>
       </c>
       <c r="C88" t="s">
-        <v>253</v>
+        <v>235</v>
       </c>
       <c r="D88" t="s">
-        <v>254</v>
+        <v>236</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B89" t="s">
-        <v>255</v>
+        <v>237</v>
       </c>
       <c r="C89" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
       <c r="D89" t="s">
-        <v>257</v>
+        <v>239</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B90" t="s">
-        <v>258</v>
+        <v>240</v>
       </c>
       <c r="C90" t="s">
-        <v>259</v>
+        <v>241</v>
       </c>
       <c r="D90" t="s">
-        <v>260</v>
+        <v>242</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B91" t="s">
-        <v>261</v>
+        <v>243</v>
       </c>
       <c r="C91" t="s">
-        <v>262</v>
+        <v>244</v>
       </c>
       <c r="D91" t="s">
-        <v>263</v>
+        <v>245</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B92" t="s">
-        <v>264</v>
+        <v>246</v>
       </c>
       <c r="C92" t="s">
-        <v>265</v>
+        <v>247</v>
       </c>
       <c r="D92" t="s">
-        <v>266</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>